<commit_message>
Updated MYS_grids_kan model - 2026-05-20 12:05
</commit_message>
<xml_diff>
--- a/VerveStacks_MYS_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_MYS_grids_kan/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_MYS_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{68ABA991-6DDA-4E9F-9948-258177114FFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{830993E3-666F-4DE4-9ECD-A524B7445F20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="940" uniqueCount="514">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="984" uniqueCount="536">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -1486,6 +1486,48 @@
     <t>elc_spv_MYS_017</t>
   </si>
   <si>
+    <t>rez_spv_MYS_018</t>
+  </si>
+  <si>
+    <t>elc_spv_MYS_018</t>
+  </si>
+  <si>
+    <t>rez_spv_MYS_019</t>
+  </si>
+  <si>
+    <t>elc_spv_MYS_019</t>
+  </si>
+  <si>
+    <t>rez_spv_MYS_020</t>
+  </si>
+  <si>
+    <t>elc_spv_MYS_020</t>
+  </si>
+  <si>
+    <t>rez_spv_MYS_021</t>
+  </si>
+  <si>
+    <t>elc_spv_MYS_021</t>
+  </si>
+  <si>
+    <t>rez_spv_MYS_022</t>
+  </si>
+  <si>
+    <t>elc_spv_MYS_022</t>
+  </si>
+  <si>
+    <t>rez_spv_MYS_023</t>
+  </si>
+  <si>
+    <t>elc_spv_MYS_023</t>
+  </si>
+  <si>
+    <t>rez_spv_MYS_024</t>
+  </si>
+  <si>
+    <t>elc_spv_MYS_024</t>
+  </si>
+  <si>
     <t>rez_won_MYS_001</t>
   </si>
   <si>
@@ -1520,6 +1562,30 @@
   </si>
   <si>
     <t>elc_won_MYS_006</t>
+  </si>
+  <si>
+    <t>rez_won_MYS_007</t>
+  </si>
+  <si>
+    <t>elc_won_MYS_007</t>
+  </si>
+  <si>
+    <t>rez_won_MYS_008</t>
+  </si>
+  <si>
+    <t>elc_won_MYS_008</t>
+  </si>
+  <si>
+    <t>rez_won_MYS_009</t>
+  </si>
+  <si>
+    <t>elc_won_MYS_009</t>
+  </si>
+  <si>
+    <t>rez_won_MYS_010</t>
+  </si>
+  <si>
+    <t>elc_won_MYS_010</t>
   </si>
   <si>
     <t>rez_wof_MYS_001</t>
@@ -2417,8 +2483,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9F39662-32C9-46E4-AE88-1C1159E2CCAE}">
-  <dimension ref="B9:E215"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0945FBAE-0686-40A1-84E9-ECB0D889E852}">
+  <dimension ref="B9:E226"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
@@ -5307,6 +5373,160 @@
         <v>513</v>
       </c>
       <c r="E215" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="216" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B216" t="s">
+        <v>514</v>
+      </c>
+      <c r="C216" t="s">
+        <v>515</v>
+      </c>
+      <c r="D216" t="s">
+        <v>515</v>
+      </c>
+      <c r="E216" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="217" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B217" t="s">
+        <v>516</v>
+      </c>
+      <c r="C217" t="s">
+        <v>517</v>
+      </c>
+      <c r="D217" t="s">
+        <v>517</v>
+      </c>
+      <c r="E217" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="218" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B218" t="s">
+        <v>518</v>
+      </c>
+      <c r="C218" t="s">
+        <v>519</v>
+      </c>
+      <c r="D218" t="s">
+        <v>519</v>
+      </c>
+      <c r="E218" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="219" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B219" t="s">
+        <v>520</v>
+      </c>
+      <c r="C219" t="s">
+        <v>521</v>
+      </c>
+      <c r="D219" t="s">
+        <v>521</v>
+      </c>
+      <c r="E219" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="220" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B220" t="s">
+        <v>522</v>
+      </c>
+      <c r="C220" t="s">
+        <v>523</v>
+      </c>
+      <c r="D220" t="s">
+        <v>523</v>
+      </c>
+      <c r="E220" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="221" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B221" t="s">
+        <v>524</v>
+      </c>
+      <c r="C221" t="s">
+        <v>525</v>
+      </c>
+      <c r="D221" t="s">
+        <v>525</v>
+      </c>
+      <c r="E221" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="222" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B222" t="s">
+        <v>526</v>
+      </c>
+      <c r="C222" t="s">
+        <v>527</v>
+      </c>
+      <c r="D222" t="s">
+        <v>527</v>
+      </c>
+      <c r="E222" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="223" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B223" t="s">
+        <v>528</v>
+      </c>
+      <c r="C223" t="s">
+        <v>529</v>
+      </c>
+      <c r="D223" t="s">
+        <v>529</v>
+      </c>
+      <c r="E223" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="224" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B224" t="s">
+        <v>530</v>
+      </c>
+      <c r="C224" t="s">
+        <v>531</v>
+      </c>
+      <c r="D224" t="s">
+        <v>531</v>
+      </c>
+      <c r="E224" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="225" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B225" t="s">
+        <v>532</v>
+      </c>
+      <c r="C225" t="s">
+        <v>533</v>
+      </c>
+      <c r="D225" t="s">
+        <v>533</v>
+      </c>
+      <c r="E225" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="226" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B226" t="s">
+        <v>534</v>
+      </c>
+      <c r="C226" t="s">
+        <v>535</v>
+      </c>
+      <c r="D226" t="s">
+        <v>535</v>
+      </c>
+      <c r="E226" t="s">
         <v>105</v>
       </c>
     </row>

</xml_diff>